<commit_message>
Add shared data intake for Volodeni Ocnita model
</commit_message>
<xml_diff>
--- a/data/finance/RENOVIT_Economic_Simulation_Model.xlsx
+++ b/data/finance/RENOVIT_Economic_Simulation_Model.xlsx
@@ -29,7 +29,13 @@
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -42,6 +48,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -53,21 +61,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Source of truth: CSV files in data/finance/simulation</t>
+          <t>CSV sources are canonical in GitHub. This workbook is regenerated from CSV for practical Excel work.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Current baseline: 10kt/year hybrid RFQ for limestone finishing materials</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Do not treat ROI/profit as confirmed before supplier RFQs and buyer prices.</t>
+          <t>Current model: Volodeni top-product raw material + Ocnita plant/logistics scenario.</t>
         </is>
       </c>
     </row>
@@ -77,6 +78,8 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -238,12 +241,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>extraction_cost_eur_per_raw_t</t>
+          <t>volodeni_limestone_cost_eur_per_raw_t</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Limestone / filler cost</t>
+          <t>Volodeni white limestone extraction</t>
         </is>
       </c>
       <c r="D6">
@@ -256,7 +259,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Partner data needed</t>
+          <t>Top product main raw material</t>
         </is>
       </c>
     </row>
@@ -268,16 +271,16 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>quarry_to_plant_transport_eur_per_raw_t</t>
+          <t>volodeni_to_ocnita_transport_eur_per_raw_t</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Internal transport / supply</t>
+          <t>Volodeni to Ocnita transport</t>
         </is>
       </c>
       <c r="D7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -286,178 +289,178 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Depends on plant location</t>
+          <t>Critical if factory is located at Ocnita</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Raw material</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>calcination_eur_per_finished_t</t>
+          <t>ocnita_limestone_cost_eur_per_raw_t</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Micronization / sorting cost</t>
+          <t>Ocnita limestone extraction</t>
         </is>
       </c>
       <c r="D8">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>EUR/t</t>
+          <t>EUR/raw t</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Former calcination field retained only for model compatibility</t>
+          <t>Volume base for decorative render and adhesive</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Raw material</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>grinding_eur_per_finished_t</t>
+          <t>ocnita_bentonite_cost_eur_per_raw_t</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dry mixing cost</t>
+          <t>Ocnita bentonite extraction / preparation</t>
         </is>
       </c>
       <c r="D9">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>EUR/t</t>
+          <t>EUR/raw t</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Mixing and dosing to target recipe</t>
+          <t>Includes working activation / preparation assumption</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Raw material</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>additives_eur_per_finished_t</t>
+          <t>weighted_raw_material_cost_eur_per_raw_t</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Additives cost</t>
+          <t>Weighted raw material cost</t>
         </is>
       </c>
       <c r="D10">
-        <v>55</v>
+        <v>5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>EUR/t</t>
+          <t>EUR/raw t</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Polymers cellulose lime/cement and performance additives</t>
+          <t>Calculated in date-initiale.html and pushed into simulation</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Processing</t>
+          <t>Raw material</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>direct_labor_eur_per_finished_t</t>
+          <t>weighted_raw_transport_eur_per_raw_t</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Direct labor</t>
+          <t>Weighted quarry to plant transport</t>
         </is>
       </c>
       <c r="D11">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>EUR/t</t>
+          <t>EUR/raw t</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Production labor</t>
+          <t>Calculated in date-initiale.html based on product recipe mix</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>bag_packaging_eur_per_bag</t>
+          <t>calcination_eur_per_finished_t</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bag and label cost</t>
+          <t>Micronization / sorting cost</t>
         </is>
       </c>
       <c r="D12">
-        <v>0.18</v>
+        <v>25</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>EUR/bag</t>
+          <t>EUR/t</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>20/25kg bag and labeling</t>
+          <t>Former calcination field retained only for model compatibility</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Logistics</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>distribution_eur_per_finished_t</t>
+          <t>grinding_eur_per_finished_t</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Distribution cost</t>
+          <t>Dry mixing cost</t>
         </is>
       </c>
       <c r="D13">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -466,28 +469,28 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Finished goods local logistics</t>
+          <t>Mixing and dosing to target recipe</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>other_variable_eur_per_finished_t</t>
+          <t>additives_eur_per_finished_t</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Other variable cost</t>
+          <t>Additives cost</t>
         </is>
       </c>
       <c r="D14">
-        <v>3</v>
+        <v>55</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -496,185 +499,305 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Spares losses and handling</t>
+          <t>Polymers cellulose lime/cement and performance additives</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Processing</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>fixed_opex_eur_per_month</t>
+          <t>direct_labor_eur_per_finished_t</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Fixed operating cost</t>
+          <t>Direct labor</t>
         </is>
       </c>
       <c r="D15">
-        <v>8000</v>
+        <v>7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>EUR/month</t>
+          <t>EUR/t</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Admin sales warehouse and base overhead</t>
+          <t>Production labor</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Working capital</t>
+          <t>Packaging</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>working_capital_months</t>
+          <t>bag_packaging_eur_per_bag</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Working capital buffer</t>
+          <t>Bag and label cost</t>
         </is>
       </c>
       <c r="D16">
-        <v>1.5</v>
+        <v>0.18</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>months</t>
+          <t>EUR/bag</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Months of variable plus fixed cost to fund</t>
+          <t>20/25kg bag and labeling</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Financing</t>
+          <t>Logistics</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>financing_enabled</t>
+          <t>distribution_eur_per_finished_t</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Financing enabled</t>
+          <t>Distribution cost</t>
         </is>
       </c>
       <c r="D17">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0/1</t>
+          <t>EUR/t</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1 means model debt service</t>
+          <t>Finished goods local logistics</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Financing</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>financed_share</t>
+          <t>other_variable_eur_per_finished_t</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Financed share of funding need</t>
+          <t>Other variable cost</t>
         </is>
       </c>
       <c r="D18">
-        <v>0.4</v>
+        <v>3</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>EUR/t</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Optional debt share</t>
+          <t>Spares losses and handling</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Financing</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>interest_rate_annual</t>
+          <t>fixed_opex_eur_per_month</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Annual interest rate</t>
+          <t>Fixed operating cost</t>
         </is>
       </c>
       <c r="D19">
-        <v>0.09</v>
+        <v>8000</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>EUR/month</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Working loan assumption</t>
+          <t>Admin sales warehouse and base overhead</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Working capital</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>working_capital_months</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Working capital buffer</t>
+        </is>
+      </c>
+      <c r="D20">
+        <v>1.5</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>months</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Months of variable plus fixed cost to fund</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Financing</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>financing_enabled</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Financing enabled</t>
+        </is>
+      </c>
+      <c r="D21">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1 means model debt service</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Financing</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>financed_share</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Financed share of funding need</t>
+        </is>
+      </c>
+      <c r="D22">
+        <v>0.4</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Optional debt share</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Financing</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>interest_rate_annual</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Annual interest rate</t>
+        </is>
+      </c>
+      <c r="D23">
+        <v>0.09</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Working loan assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Financing</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>loan_term_years</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Loan term</t>
         </is>
       </c>
-      <c r="D20">
+      <c r="D24">
         <v>5</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>years</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>Optional debt term</t>
         </is>
@@ -686,6 +809,8 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -879,6 +1004,8 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:E49"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2113,6 +2240,8 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G4"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2212,7 +2341,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.00</v>
+        <v>0</v>
       </c>
       <c r="C4">
         <v>0.08</v>
@@ -2238,6 +2367,8 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -2613,6 +2744,8 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:N15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3700,6 +3833,8 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F7"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -3821,7 +3956,7 @@
         <v>1.20</v>
       </c>
       <c r="C5">
-        <v>1.00</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <v>0.90</v>
@@ -3895,18 +4030,41 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Decision rule</t>
+          <t>Decision</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GO only after: validated wholesale prices, tested recipe, supplier RFQs, full CAPEX with install/commissioning, realistic utilization.</t>
+          <t>Factory working assumption: Ocnita, because of railway node.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Top product raw material: Volodeni white limestone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Critical input: Volodeni -&gt; Ocnita transport EUR/t.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Use date-initiale.html as browser source of truth for live assumptions.</t>
         </is>
       </c>
     </row>

</xml_diff>